<commit_message>
Header agrandado con logo texto blanco + header Excel del quote actualizado
</commit_message>
<xml_diff>
--- a/backend/app/quotes/services/assets/quote_template.xlsx
+++ b/backend/app/quotes/services/assets/quote_template.xlsx
@@ -3,13 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_quote" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </externalReferences>
   <definedNames>
-    <definedName name="ClientList">_CLIENTS!$A$1:$A$996</definedName>
+    <definedName name="ClientList">[1]_CLIENTS!$A$1:$A$996</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -50,14 +53,6 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -79,7 +74,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -109,17 +104,6 @@
       <right style="thin">
         <color theme="0"/>
       </right>
-      <top style="thin">
-        <color theme="0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0"/>
-      </left>
-      <right/>
       <top style="thin">
         <color theme="0"/>
       </top>
@@ -363,552 +347,104 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="1"/>
-        <extend val="0"/>
-        <sz val="12"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center"/>
-      <border outline="0">
-        <left style="thin">
-          <color theme="1"/>
-        </left>
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <color theme="1"/>
-        <sz val="11"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-  </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Стиль таблицы 1" pivot="0" count="0"/>
   </tableStyles>
@@ -981,6 +517,49 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="933450"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="_CLIENTS"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1305,22 +884,22 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K59"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="6.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="11" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="9.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="34.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="18.7109375" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="20.140625" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="17.7109375" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="18" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="19.42578125" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="21.7109375" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="12" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="6.6640625" bestFit="1" customWidth="1" style="34" min="1" max="1"/>
+    <col width="11" bestFit="1" customWidth="1" style="34" min="2" max="2"/>
+    <col width="9.33203125" bestFit="1" customWidth="1" style="34" min="3" max="3"/>
+    <col width="34.5546875" bestFit="1" customWidth="1" style="34" min="4" max="4"/>
+    <col width="18.6640625" bestFit="1" customWidth="1" style="34" min="5" max="5"/>
+    <col width="20.109375" bestFit="1" customWidth="1" style="34" min="6" max="6"/>
+    <col width="17.6640625" bestFit="1" customWidth="1" style="34" min="7" max="7"/>
+    <col width="18" bestFit="1" customWidth="1" style="34" min="8" max="8"/>
+    <col width="19.44140625" bestFit="1" customWidth="1" style="34" min="9" max="9"/>
+    <col width="21.6640625" bestFit="1" customWidth="1" style="34" min="10" max="10"/>
+    <col width="12" bestFit="1" customWidth="1" style="34" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1" s="34">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
@@ -1332,17 +911,10 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="1" t="n"/>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="41" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="B2" s="42" t="n"/>
-      <c r="C2" s="43" t="n"/>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>SEVEN ROADS GROUP</t>
-        </is>
-      </c>
+    <row r="2" ht="15.75" customHeight="1" s="34">
+      <c r="A2" s="30" t="n"/>
+      <c r="B2" s="31" t="n"/>
+      <c r="C2" s="32" t="n"/>
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
@@ -1354,12 +926,12 @@
       </c>
       <c r="J2" s="6" t="n"/>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="44" t="n"/>
-      <c r="C3" s="45" t="n"/>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>8109 NW 29TH STREET</t>
+    <row r="3" ht="15.75" customHeight="1" s="34">
+      <c r="A3" s="33" t="n"/>
+      <c r="C3" s="35" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>SEVEN ROADS GROUP</t>
         </is>
       </c>
       <c r="E3" s="3" t="n"/>
@@ -1376,12 +948,12 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="44" t="n"/>
-      <c r="C4" s="45" t="n"/>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>MIAMI FL 33122</t>
+    <row r="4" ht="15.75" customHeight="1" s="34">
+      <c r="A4" s="33" t="n"/>
+      <c r="C4" s="35" t="n"/>
+      <c r="D4" s="39" t="inlineStr">
+        <is>
+          <t>OFFICE: 305.377.8997</t>
         </is>
       </c>
       <c r="E4" s="7" t="n"/>
@@ -1399,12 +971,12 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="44" t="n"/>
-      <c r="C5" s="45" t="n"/>
+    <row r="5" ht="15.75" customHeight="1" s="34">
+      <c r="A5" s="33" t="n"/>
+      <c r="C5" s="35" t="n"/>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>+1 (305) 377-8997</t>
+          <t>PARTS@SEVENROADSGROUP.COM</t>
         </is>
       </c>
       <c r="E5" s="7" t="n"/>
@@ -1418,12 +990,12 @@
       </c>
       <c r="J5" s="5" t="n"/>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="44" t="n"/>
-      <c r="C6" s="45" t="n"/>
+    <row r="6" ht="15.75" customHeight="1" s="34">
+      <c r="A6" s="33" t="n"/>
+      <c r="C6" s="35" t="n"/>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>PARTS@SEVENROADSGROUP.COM</t>
+          <t>WWW.SEVENROADSGROUP.COM</t>
         </is>
       </c>
       <c r="E6" s="7" t="n"/>
@@ -1433,15 +1005,10 @@
       <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="n"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="46" t="n"/>
-      <c r="B7" s="47" t="n"/>
-      <c r="C7" s="48" t="n"/>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>WWW.SEVENROADSGROUP.COM</t>
-        </is>
-      </c>
+    <row r="7" ht="15.75" customHeight="1" s="34">
+      <c r="A7" s="36" t="n"/>
+      <c r="B7" s="37" t="n"/>
+      <c r="C7" s="38" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="1" t="n"/>
       <c r="G7" s="1" t="n"/>
@@ -1449,7 +1016,7 @@
       <c r="I7" s="1" t="n"/>
       <c r="J7" s="1" t="n"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" ht="15.75" customHeight="1" s="34">
       <c r="A8" s="1" t="n"/>
       <c r="B8" s="1" t="n"/>
       <c r="C8" s="1" t="n"/>
@@ -1461,7 +1028,7 @@
       <c r="I8" s="1" t="n"/>
       <c r="J8" s="1" t="n"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" ht="15.75" customHeight="1" s="34">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="n"/>
@@ -1473,7 +1040,7 @@
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="n"/>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" ht="15.75" customHeight="1" s="34">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>#</t>
@@ -1530,14 +1097,14 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" ht="15.75" customHeight="1" s="34">
       <c r="A11" s="9" t="n"/>
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9" t="n"/>
-      <c r="F11" s="49" t="n"/>
-      <c r="G11" s="50">
+      <c r="F11" s="40" t="n"/>
+      <c r="G11" s="41">
         <f>SUM(F11*C11)</f>
         <v/>
       </c>
@@ -1549,14 +1116,14 @@
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="9" t="n"/>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" ht="15.75" customHeight="1" s="34">
       <c r="A12" s="9" t="n"/>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
-      <c r="F12" s="49" t="n"/>
-      <c r="G12" s="50">
+      <c r="F12" s="40" t="n"/>
+      <c r="G12" s="41">
         <f>SUM(F12*C12)</f>
         <v/>
       </c>
@@ -1568,14 +1135,14 @@
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="9" t="n"/>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" ht="15.75" customHeight="1" s="34">
       <c r="A13" s="9" t="n"/>
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="9" t="n"/>
-      <c r="F13" s="49" t="n"/>
-      <c r="G13" s="50">
+      <c r="F13" s="40" t="n"/>
+      <c r="G13" s="41">
         <f>SUM(F13*C13)</f>
         <v/>
       </c>
@@ -1587,14 +1154,14 @@
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="n"/>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" ht="15.75" customHeight="1" s="34">
       <c r="A14" s="9" t="n"/>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9" t="n"/>
-      <c r="F14" s="49" t="n"/>
-      <c r="G14" s="50">
+      <c r="F14" s="40" t="n"/>
+      <c r="G14" s="41">
         <f>SUM(F14*C14)</f>
         <v/>
       </c>
@@ -1606,14 +1173,14 @@
       <c r="J14" s="9" t="n"/>
       <c r="K14" s="9" t="n"/>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" ht="15.75" customHeight="1" s="34">
       <c r="A15" s="9" t="n"/>
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="9" t="n"/>
-      <c r="F15" s="49" t="n"/>
-      <c r="G15" s="50">
+      <c r="F15" s="40" t="n"/>
+      <c r="G15" s="41">
         <f>SUM(F15*C15)</f>
         <v/>
       </c>
@@ -1625,14 +1192,14 @@
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
+    <row r="16" ht="15.75" customHeight="1" s="34">
       <c r="A16" s="9" t="n"/>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="9" t="n"/>
-      <c r="F16" s="49" t="n"/>
-      <c r="G16" s="50">
+      <c r="F16" s="40" t="n"/>
+      <c r="G16" s="41">
         <f>SUM(F16*C16)</f>
         <v/>
       </c>
@@ -1644,14 +1211,14 @@
       <c r="J16" s="9" t="n"/>
       <c r="K16" s="9" t="n"/>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" ht="15.75" customHeight="1" s="34">
       <c r="A17" s="9" t="n"/>
       <c r="B17" s="9" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="9" t="n"/>
-      <c r="F17" s="49" t="n"/>
-      <c r="G17" s="50">
+      <c r="F17" s="40" t="n"/>
+      <c r="G17" s="41">
         <f>SUM(F17*C17)</f>
         <v/>
       </c>
@@ -1663,14 +1230,14 @@
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="9" t="n"/>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
+    <row r="18" ht="15.75" customHeight="1" s="34">
       <c r="A18" s="9" t="n"/>
       <c r="B18" s="9" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="9" t="n"/>
-      <c r="F18" s="49" t="n"/>
-      <c r="G18" s="50">
+      <c r="F18" s="40" t="n"/>
+      <c r="G18" s="41">
         <f>SUM(F18*C18)</f>
         <v/>
       </c>
@@ -1682,14 +1249,14 @@
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="9" t="n"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="15.75" customHeight="1" s="34">
       <c r="A19" s="9" t="n"/>
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="9" t="n"/>
-      <c r="F19" s="49" t="n"/>
-      <c r="G19" s="50">
+      <c r="F19" s="40" t="n"/>
+      <c r="G19" s="41">
         <f>SUM(F19*C19)</f>
         <v/>
       </c>
@@ -1701,14 +1268,14 @@
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="9" t="n"/>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1" s="34">
       <c r="A20" s="9" t="n"/>
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="9" t="n"/>
-      <c r="F20" s="49" t="n"/>
-      <c r="G20" s="50">
+      <c r="F20" s="40" t="n"/>
+      <c r="G20" s="41">
         <f>SUM(F20*C20)</f>
         <v/>
       </c>
@@ -1720,14 +1287,14 @@
       <c r="J20" s="9" t="n"/>
       <c r="K20" s="9" t="n"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1" s="34">
       <c r="A21" s="9" t="n"/>
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="9" t="n"/>
-      <c r="F21" s="49" t="n"/>
-      <c r="G21" s="50">
+      <c r="F21" s="40" t="n"/>
+      <c r="G21" s="41">
         <f>SUM(F21*C21)</f>
         <v/>
       </c>
@@ -1739,14 +1306,14 @@
       <c r="J21" s="9" t="n"/>
       <c r="K21" s="9" t="n"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1" s="34">
       <c r="A22" s="9" t="n"/>
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="9" t="n"/>
-      <c r="F22" s="49" t="n"/>
-      <c r="G22" s="50">
+      <c r="F22" s="40" t="n"/>
+      <c r="G22" s="41">
         <f>SUM(F22*C22)</f>
         <v/>
       </c>
@@ -1758,14 +1325,14 @@
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="9" t="n"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1" s="34">
       <c r="A23" s="9" t="n"/>
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
-      <c r="F23" s="49" t="n"/>
-      <c r="G23" s="50">
+      <c r="F23" s="40" t="n"/>
+      <c r="G23" s="41">
         <f>SUM(F23*C23)</f>
         <v/>
       </c>
@@ -1777,14 +1344,14 @@
       <c r="J23" s="9" t="n"/>
       <c r="K23" s="9" t="n"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1" s="34">
       <c r="A24" s="9" t="n"/>
       <c r="B24" s="9" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
-      <c r="F24" s="49" t="n"/>
-      <c r="G24" s="50">
+      <c r="F24" s="40" t="n"/>
+      <c r="G24" s="41">
         <f>SUM(F24*C24)</f>
         <v/>
       </c>
@@ -1796,14 +1363,14 @@
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="9" t="n"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" ht="15.75" customHeight="1" s="34">
       <c r="A25" s="9" t="n"/>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n"/>
-      <c r="F25" s="49" t="n"/>
-      <c r="G25" s="50">
+      <c r="F25" s="40" t="n"/>
+      <c r="G25" s="41">
         <f>SUM(F25*C25)</f>
         <v/>
       </c>
@@ -1815,14 +1382,14 @@
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="9" t="n"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" ht="15.75" customHeight="1" s="34">
       <c r="A26" s="9" t="n"/>
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
-      <c r="F26" s="49" t="n"/>
-      <c r="G26" s="50">
+      <c r="F26" s="40" t="n"/>
+      <c r="G26" s="41">
         <f>SUM(F26*C26)</f>
         <v/>
       </c>
@@ -1834,14 +1401,14 @@
       <c r="J26" s="9" t="n"/>
       <c r="K26" s="9" t="n"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" ht="15.75" customHeight="1" s="34">
       <c r="A27" s="9" t="n"/>
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
-      <c r="F27" s="49" t="n"/>
-      <c r="G27" s="50">
+      <c r="F27" s="40" t="n"/>
+      <c r="G27" s="41">
         <f>SUM(F27*C27)</f>
         <v/>
       </c>
@@ -1853,14 +1420,14 @@
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="9" t="n"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="15.75" customHeight="1" s="34">
       <c r="A28" s="9" t="n"/>
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
-      <c r="F28" s="49" t="n"/>
-      <c r="G28" s="50">
+      <c r="F28" s="40" t="n"/>
+      <c r="G28" s="41">
         <f>SUM(F28*C28)</f>
         <v/>
       </c>
@@ -1872,14 +1439,14 @@
       <c r="J28" s="9" t="n"/>
       <c r="K28" s="9" t="n"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1" s="34">
       <c r="A29" s="9" t="n"/>
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
-      <c r="F29" s="49" t="n"/>
-      <c r="G29" s="50">
+      <c r="F29" s="40" t="n"/>
+      <c r="G29" s="41">
         <f>SUM(F29*C29)</f>
         <v/>
       </c>
@@ -1891,14 +1458,14 @@
       <c r="J29" s="9" t="n"/>
       <c r="K29" s="9" t="n"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" ht="15.75" customHeight="1" s="34">
       <c r="A30" s="9" t="n"/>
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="9" t="n"/>
-      <c r="F30" s="49" t="n"/>
-      <c r="G30" s="50">
+      <c r="F30" s="40" t="n"/>
+      <c r="G30" s="41">
         <f>SUM(F30*C30)</f>
         <v/>
       </c>
@@ -1910,14 +1477,14 @@
       <c r="J30" s="9" t="n"/>
       <c r="K30" s="9" t="n"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1" s="34">
       <c r="A31" s="9" t="n"/>
       <c r="B31" s="9" t="n"/>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="9" t="n"/>
-      <c r="F31" s="49" t="n"/>
-      <c r="G31" s="50">
+      <c r="F31" s="40" t="n"/>
+      <c r="G31" s="41">
         <f>SUM(F31*C31)</f>
         <v/>
       </c>
@@ -1929,14 +1496,14 @@
       <c r="J31" s="9" t="n"/>
       <c r="K31" s="9" t="n"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="15.75" customHeight="1" s="34">
       <c r="A32" s="9" t="n"/>
       <c r="B32" s="9" t="n"/>
       <c r="C32" s="15" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="9" t="n"/>
-      <c r="F32" s="49" t="n"/>
-      <c r="G32" s="50">
+      <c r="F32" s="40" t="n"/>
+      <c r="G32" s="41">
         <f>SUM(F32*C32)</f>
         <v/>
       </c>
@@ -1948,14 +1515,14 @@
       <c r="J32" s="9" t="n"/>
       <c r="K32" s="9" t="n"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="15.75" customHeight="1" s="34">
       <c r="A33" s="9" t="n"/>
       <c r="B33" s="9" t="n"/>
       <c r="C33" s="15" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="9" t="n"/>
-      <c r="F33" s="49" t="n"/>
-      <c r="G33" s="50">
+      <c r="F33" s="40" t="n"/>
+      <c r="G33" s="41">
         <f>SUM(F33*C33)</f>
         <v/>
       </c>
@@ -1967,14 +1534,14 @@
       <c r="J33" s="9" t="n"/>
       <c r="K33" s="9" t="n"/>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" ht="15.75" customHeight="1" s="34">
       <c r="A34" s="9" t="n"/>
       <c r="B34" s="9" t="n"/>
       <c r="C34" s="15" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="9" t="n"/>
-      <c r="F34" s="49" t="n"/>
-      <c r="G34" s="50">
+      <c r="F34" s="40" t="n"/>
+      <c r="G34" s="41">
         <f>SUM(F34*C34)</f>
         <v/>
       </c>
@@ -1986,14 +1553,14 @@
       <c r="J34" s="9" t="n"/>
       <c r="K34" s="9" t="n"/>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" ht="15.75" customHeight="1" s="34">
       <c r="A35" s="9" t="n"/>
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="15" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="9" t="n"/>
-      <c r="F35" s="49" t="n"/>
-      <c r="G35" s="50">
+      <c r="F35" s="40" t="n"/>
+      <c r="G35" s="41">
         <f>SUM(F35*C35)</f>
         <v/>
       </c>
@@ -2005,14 +1572,14 @@
       <c r="J35" s="9" t="n"/>
       <c r="K35" s="9" t="n"/>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" ht="15.75" customHeight="1" s="34">
       <c r="A36" s="9" t="n"/>
       <c r="B36" s="9" t="n"/>
       <c r="C36" s="15" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="9" t="n"/>
-      <c r="F36" s="49" t="n"/>
-      <c r="G36" s="50">
+      <c r="F36" s="40" t="n"/>
+      <c r="G36" s="41">
         <f>SUM(F36*C36)</f>
         <v/>
       </c>
@@ -2024,14 +1591,14 @@
       <c r="J36" s="9" t="n"/>
       <c r="K36" s="9" t="n"/>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="15.75" customHeight="1" s="34">
       <c r="A37" s="9" t="n"/>
       <c r="B37" s="9" t="n"/>
       <c r="C37" s="15" t="n"/>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="9" t="n"/>
-      <c r="F37" s="49" t="n"/>
-      <c r="G37" s="50">
+      <c r="F37" s="40" t="n"/>
+      <c r="G37" s="41">
         <f>SUM(F37*C37)</f>
         <v/>
       </c>
@@ -2043,14 +1610,14 @@
       <c r="J37" s="9" t="n"/>
       <c r="K37" s="9" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="15.75" customHeight="1" s="34">
       <c r="A38" s="9" t="n"/>
       <c r="B38" s="9" t="n"/>
       <c r="C38" s="15" t="n"/>
       <c r="D38" s="9" t="n"/>
       <c r="E38" s="9" t="n"/>
-      <c r="F38" s="49" t="n"/>
-      <c r="G38" s="50">
+      <c r="F38" s="40" t="n"/>
+      <c r="G38" s="41">
         <f>SUM(F38*C38)</f>
         <v/>
       </c>
@@ -2062,14 +1629,14 @@
       <c r="J38" s="9" t="n"/>
       <c r="K38" s="9" t="n"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="15.75" customHeight="1" s="34">
       <c r="A39" s="9" t="n"/>
       <c r="B39" s="9" t="n"/>
       <c r="C39" s="15" t="n"/>
       <c r="D39" s="9" t="n"/>
       <c r="E39" s="9" t="n"/>
-      <c r="F39" s="49" t="n"/>
-      <c r="G39" s="50">
+      <c r="F39" s="40" t="n"/>
+      <c r="G39" s="41">
         <f>SUM(F39*C39)</f>
         <v/>
       </c>
@@ -2081,14 +1648,14 @@
       <c r="J39" s="9" t="n"/>
       <c r="K39" s="9" t="n"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" ht="15.75" customHeight="1" s="34">
       <c r="A40" s="9" t="n"/>
       <c r="B40" s="9" t="n"/>
       <c r="C40" s="15" t="n"/>
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
-      <c r="F40" s="49" t="n"/>
-      <c r="G40" s="50">
+      <c r="F40" s="40" t="n"/>
+      <c r="G40" s="41">
         <f>SUM(F40*C40)</f>
         <v/>
       </c>
@@ -2100,14 +1667,14 @@
       <c r="J40" s="9" t="n"/>
       <c r="K40" s="9" t="n"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="15.75" customHeight="1" s="34">
       <c r="A41" s="9" t="n"/>
       <c r="B41" s="9" t="n"/>
       <c r="C41" s="15" t="n"/>
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="9" t="n"/>
-      <c r="F41" s="49" t="n"/>
-      <c r="G41" s="50">
+      <c r="F41" s="40" t="n"/>
+      <c r="G41" s="41">
         <f>SUM(F41*C41)</f>
         <v/>
       </c>
@@ -2119,14 +1686,14 @@
       <c r="J41" s="9" t="n"/>
       <c r="K41" s="9" t="n"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" ht="15.75" customHeight="1" s="34">
       <c r="A42" s="9" t="n"/>
       <c r="B42" s="9" t="n"/>
       <c r="C42" s="15" t="n"/>
       <c r="D42" s="9" t="n"/>
       <c r="E42" s="9" t="n"/>
-      <c r="F42" s="49" t="n"/>
-      <c r="G42" s="50">
+      <c r="F42" s="40" t="n"/>
+      <c r="G42" s="41">
         <f>SUM(F42*C42)</f>
         <v/>
       </c>
@@ -2138,14 +1705,14 @@
       <c r="J42" s="9" t="n"/>
       <c r="K42" s="9" t="n"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" ht="15.75" customHeight="1" s="34">
       <c r="A43" s="9" t="n"/>
       <c r="B43" s="9" t="n"/>
       <c r="C43" s="15" t="n"/>
       <c r="D43" s="9" t="n"/>
       <c r="E43" s="9" t="n"/>
-      <c r="F43" s="49" t="n"/>
-      <c r="G43" s="50">
+      <c r="F43" s="40" t="n"/>
+      <c r="G43" s="41">
         <f>SUM(F43*C43)</f>
         <v/>
       </c>
@@ -2157,14 +1724,14 @@
       <c r="J43" s="9" t="n"/>
       <c r="K43" s="9" t="n"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="15.75" customHeight="1" s="34">
       <c r="A44" s="9" t="n"/>
       <c r="B44" s="9" t="n"/>
       <c r="C44" s="15" t="n"/>
       <c r="D44" s="9" t="n"/>
       <c r="E44" s="9" t="n"/>
-      <c r="F44" s="49" t="n"/>
-      <c r="G44" s="50">
+      <c r="F44" s="40" t="n"/>
+      <c r="G44" s="41">
         <f>SUM(F44*C44)</f>
         <v/>
       </c>
@@ -2176,14 +1743,14 @@
       <c r="J44" s="9" t="n"/>
       <c r="K44" s="9" t="n"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="15.75" customHeight="1" s="34">
       <c r="A45" s="9" t="n"/>
       <c r="B45" s="9" t="n"/>
       <c r="C45" s="15" t="n"/>
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="9" t="n"/>
-      <c r="F45" s="49" t="n"/>
-      <c r="G45" s="50">
+      <c r="F45" s="40" t="n"/>
+      <c r="G45" s="41">
         <f>SUM(F45*C45)</f>
         <v/>
       </c>
@@ -2195,14 +1762,14 @@
       <c r="J45" s="9" t="n"/>
       <c r="K45" s="9" t="n"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" ht="15.75" customHeight="1" s="34">
       <c r="A46" s="9" t="n"/>
       <c r="B46" s="9" t="n"/>
       <c r="C46" s="15" t="n"/>
       <c r="D46" s="9" t="n"/>
       <c r="E46" s="9" t="n"/>
-      <c r="F46" s="49" t="n"/>
-      <c r="G46" s="50">
+      <c r="F46" s="40" t="n"/>
+      <c r="G46" s="41">
         <f>SUM(F46*C46)</f>
         <v/>
       </c>
@@ -2214,14 +1781,14 @@
       <c r="J46" s="9" t="n"/>
       <c r="K46" s="9" t="n"/>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" ht="15.75" customHeight="1" s="34">
       <c r="A47" s="9" t="n"/>
       <c r="B47" s="9" t="n"/>
       <c r="C47" s="15" t="n"/>
       <c r="D47" s="9" t="n"/>
       <c r="E47" s="9" t="n"/>
-      <c r="F47" s="49" t="n"/>
-      <c r="G47" s="50">
+      <c r="F47" s="40" t="n"/>
+      <c r="G47" s="41">
         <f>SUM(F47*C47)</f>
         <v/>
       </c>
@@ -2233,14 +1800,14 @@
       <c r="J47" s="9" t="n"/>
       <c r="K47" s="9" t="n"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" ht="15.75" customHeight="1" s="34">
       <c r="A48" s="9" t="n"/>
       <c r="B48" s="9" t="n"/>
       <c r="C48" s="15" t="n"/>
       <c r="D48" s="9" t="n"/>
       <c r="E48" s="9" t="n"/>
-      <c r="F48" s="49" t="n"/>
-      <c r="G48" s="50">
+      <c r="F48" s="40" t="n"/>
+      <c r="G48" s="41">
         <f>SUM(F48*C48)</f>
         <v/>
       </c>
@@ -2252,14 +1819,14 @@
       <c r="J48" s="9" t="n"/>
       <c r="K48" s="9" t="n"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" ht="15.75" customHeight="1" s="34">
       <c r="A49" s="9" t="n"/>
       <c r="B49" s="9" t="n"/>
       <c r="C49" s="15" t="n"/>
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="9" t="n"/>
-      <c r="F49" s="49" t="n"/>
-      <c r="G49" s="50">
+      <c r="F49" s="40" t="n"/>
+      <c r="G49" s="41">
         <f>SUM(F49*C49)</f>
         <v/>
       </c>
@@ -2271,14 +1838,14 @@
       <c r="J49" s="9" t="n"/>
       <c r="K49" s="9" t="n"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" ht="15.75" customHeight="1" s="34">
       <c r="A50" s="9" t="n"/>
       <c r="B50" s="9" t="n"/>
       <c r="C50" s="15" t="n"/>
       <c r="D50" s="9" t="n"/>
       <c r="E50" s="9" t="n"/>
-      <c r="F50" s="49" t="n"/>
-      <c r="G50" s="50">
+      <c r="F50" s="40" t="n"/>
+      <c r="G50" s="41">
         <f>SUM(F50*C50)</f>
         <v/>
       </c>
@@ -2290,14 +1857,14 @@
       <c r="J50" s="9" t="n"/>
       <c r="K50" s="9" t="n"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" ht="15.75" customHeight="1" s="34">
       <c r="A51" s="9" t="n"/>
       <c r="B51" s="9" t="n"/>
       <c r="C51" s="15" t="n"/>
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="9" t="n"/>
-      <c r="F51" s="49" t="n"/>
-      <c r="G51" s="50">
+      <c r="F51" s="40" t="n"/>
+      <c r="G51" s="41">
         <f>SUM(F51*C51)</f>
         <v/>
       </c>
@@ -2309,14 +1876,14 @@
       <c r="J51" s="9" t="n"/>
       <c r="K51" s="9" t="n"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" ht="15.75" customHeight="1" s="34">
       <c r="A52" s="9" t="n"/>
       <c r="B52" s="9" t="n"/>
       <c r="C52" s="15" t="n"/>
       <c r="D52" s="9" t="n"/>
       <c r="E52" s="9" t="n"/>
-      <c r="F52" s="49" t="n"/>
-      <c r="G52" s="50">
+      <c r="F52" s="40" t="n"/>
+      <c r="G52" s="41">
         <f>SUM(F52*C52)</f>
         <v/>
       </c>
@@ -2328,14 +1895,14 @@
       <c r="J52" s="9" t="n"/>
       <c r="K52" s="9" t="n"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" ht="15.75" customHeight="1" s="34">
       <c r="A53" s="9" t="n"/>
       <c r="B53" s="9" t="n"/>
       <c r="C53" s="15" t="n"/>
       <c r="D53" s="9" t="n"/>
       <c r="E53" s="9" t="n"/>
-      <c r="F53" s="49" t="n"/>
-      <c r="G53" s="50">
+      <c r="F53" s="40" t="n"/>
+      <c r="G53" s="41">
         <f>SUM(F53*C53)</f>
         <v/>
       </c>
@@ -2347,14 +1914,14 @@
       <c r="J53" s="9" t="n"/>
       <c r="K53" s="9" t="n"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" ht="15.75" customHeight="1" s="34">
       <c r="A54" s="9" t="n"/>
       <c r="B54" s="9" t="n"/>
       <c r="C54" s="15" t="n"/>
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="9" t="n"/>
-      <c r="F54" s="49" t="n"/>
-      <c r="G54" s="50">
+      <c r="F54" s="40" t="n"/>
+      <c r="G54" s="41">
         <f>SUM(F54*C54)</f>
         <v/>
       </c>
@@ -2366,14 +1933,14 @@
       <c r="J54" s="9" t="n"/>
       <c r="K54" s="9" t="n"/>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" ht="15.75" customHeight="1" s="34">
       <c r="A55" s="9" t="n"/>
       <c r="B55" s="9" t="n"/>
       <c r="C55" s="15" t="n"/>
       <c r="D55" s="9" t="n"/>
       <c r="E55" s="9" t="n"/>
-      <c r="F55" s="49" t="n"/>
-      <c r="G55" s="50">
+      <c r="F55" s="40" t="n"/>
+      <c r="G55" s="41">
         <f>SUM(F55*C55)</f>
         <v/>
       </c>
@@ -2385,14 +1952,14 @@
       <c r="J55" s="9" t="n"/>
       <c r="K55" s="9" t="n"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
+    <row r="56" ht="15.75" customHeight="1" s="34">
       <c r="A56" s="9" t="n"/>
       <c r="B56" s="9" t="n"/>
       <c r="C56" s="15" t="n"/>
       <c r="D56" s="9" t="n"/>
       <c r="E56" s="9" t="n"/>
-      <c r="F56" s="49" t="n"/>
-      <c r="G56" s="50">
+      <c r="F56" s="40" t="n"/>
+      <c r="G56" s="41">
         <f>SUM(F56*C56)</f>
         <v/>
       </c>
@@ -2404,18 +1971,18 @@
       <c r="J56" s="19" t="n"/>
       <c r="K56" s="19" t="n"/>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" ht="15.75" customHeight="1" s="34">
       <c r="A57" s="12" t="n"/>
       <c r="B57" s="12" t="n"/>
       <c r="C57" s="12" t="n"/>
       <c r="D57" s="12" t="n"/>
       <c r="E57" s="13" t="n"/>
-      <c r="F57" s="36" t="inlineStr">
+      <c r="F57" s="24" t="inlineStr">
         <is>
           <t>Total (USD)</t>
         </is>
       </c>
-      <c r="G57" s="51">
+      <c r="G57" s="42">
         <f>SUM(G11:G56)</f>
         <v/>
       </c>
@@ -2431,24 +1998,24 @@
       <c r="J57" s="21" t="n"/>
       <c r="K57" s="20" t="n"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" ht="15.75" customHeight="1" s="34">
       <c r="A58" s="1" t="n"/>
       <c r="B58" s="1" t="n"/>
       <c r="C58" s="1" t="n"/>
       <c r="D58" s="1" t="n"/>
-      <c r="E58" s="34" t="n"/>
-      <c r="F58" s="39" t="inlineStr">
+      <c r="E58" s="22" t="n"/>
+      <c r="F58" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">Shipping cost (USD) </t>
         </is>
       </c>
-      <c r="G58" s="52" t="n"/>
-      <c r="H58" s="35" t="n"/>
+      <c r="G58" s="43" t="n"/>
+      <c r="H58" s="23" t="n"/>
       <c r="I58" s="14" t="n"/>
       <c r="J58" s="14" t="n"/>
     </row>
-    <row r="59" ht="186" customHeight="1">
-      <c r="A59" s="32" t="inlineStr">
+    <row r="59" ht="186" customHeight="1" s="34">
+      <c r="A59" s="28" t="inlineStr">
         <is>
           <t>Payment options:
 1) Wire transfer (TT transfer)/ ACH Payment
@@ -2461,14 +2028,14 @@
 Debido a las regulaciones de fabricación, si la pieza se exporta fuera de los Estados Unidos, Seven Roads Group no ofrecerá ninguna garantía.</t>
         </is>
       </c>
-      <c r="B59" s="53" t="n"/>
-      <c r="C59" s="53" t="n"/>
-      <c r="D59" s="53" t="n"/>
-      <c r="E59" s="53" t="n"/>
-      <c r="F59" s="53" t="n"/>
-      <c r="G59" s="53" t="n"/>
-      <c r="H59" s="53" t="n"/>
-      <c r="I59" s="53" t="n"/>
+      <c r="B59" s="29" t="n"/>
+      <c r="C59" s="29" t="n"/>
+      <c r="D59" s="29" t="n"/>
+      <c r="E59" s="29" t="n"/>
+      <c r="F59" s="29" t="n"/>
+      <c r="G59" s="29" t="n"/>
+      <c r="H59" s="29" t="n"/>
+      <c r="I59" s="29" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2481,5 +2048,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>